<commit_message>
Add Cycle Data Excel
</commit_message>
<xml_diff>
--- a/Data/GasTurb/constraintPerformanceData.xlsx
+++ b/Data/GasTurb/constraintPerformanceData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bendelej\Desktop\AE 440\Detail-Design\Data\GasTurb\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\clardyj\Desktop\AERO440\Detail-Design\Data\GasTurb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE34E408-4B66-4720-A3E8-CD5C56BA8958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5F530F16-6A7D-419F-A4BF-7843A9D9AC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B0EB3282-DFD5-48BB-B3F6-C3DE2811492B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8E8E9A7-5DA1-4ED5-A8B4-C4B5FE86D3E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
     <t>CEILING</t>
   </si>
   <si>
-    <t>TOLDG</t>
+    <t>RTO</t>
   </si>
   <si>
     <t>SLS</t>
@@ -985,7 +985,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B258ACE5-C1EC-45F5-B1CC-0E253BD4EF5A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96CA2823-B41B-4E07-9BEB-BAA571A63372}">
   <dimension ref="A2:H176"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1021,22 +1021,22 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>13.1</v>
+        <v>34.1</v>
       </c>
       <c r="D3">
-        <v>13.1</v>
+        <v>30.1</v>
       </c>
       <c r="E3">
-        <v>53.1</v>
+        <v>52.1</v>
       </c>
       <c r="F3">
         <v>19.100000000000001</v>
       </c>
       <c r="G3">
-        <v>35.1</v>
+        <v>49.1</v>
       </c>
       <c r="H3">
-        <v>34.1</v>
+        <v>84.1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1122,7 +1122,7 @@
         <v>0.63</v>
       </c>
       <c r="D7">
-        <v>0.63</v>
+        <v>0.8</v>
       </c>
       <c r="E7">
         <v>0.7</v>
@@ -1197,22 +1197,22 @@
         <v>19</v>
       </c>
       <c r="C10">
-        <v>6.9813200000000002</v>
+        <v>5.5002500000000003</v>
       </c>
       <c r="D10">
-        <v>7.0739000000000001</v>
+        <v>5.9244599999999998</v>
       </c>
       <c r="E10">
-        <v>16.544</v>
+        <v>14.2888</v>
       </c>
       <c r="F10">
-        <v>5.9405599999999996</v>
+        <v>4.8992000000000004</v>
       </c>
       <c r="G10">
-        <v>24.15</v>
+        <v>18.182099999999998</v>
       </c>
       <c r="H10">
-        <v>27.268699999999999</v>
+        <v>22.3508</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1223,22 +1223,22 @@
         <v>19</v>
       </c>
       <c r="C11">
-        <v>10.621499999999999</v>
+        <v>8.8069799999999994</v>
       </c>
       <c r="D11">
-        <v>10.7287</v>
+        <v>10.697800000000001</v>
       </c>
       <c r="E11">
-        <v>29.053799999999999</v>
+        <v>26.159500000000001</v>
       </c>
       <c r="F11">
-        <v>10.1799</v>
+        <v>8.8012200000000007</v>
       </c>
       <c r="G11">
-        <v>28.247399999999999</v>
+        <v>21.864999999999998</v>
       </c>
       <c r="H11">
-        <v>27.268699999999999</v>
+        <v>22.3508</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1249,22 +1249,22 @@
         <v>22</v>
       </c>
       <c r="C12">
-        <v>20.091799999999999</v>
+        <v>19.959599999999998</v>
       </c>
       <c r="D12">
-        <v>20.157499999999999</v>
+        <v>21.3856</v>
       </c>
       <c r="E12">
-        <v>21.8428</v>
+        <v>21.9009</v>
       </c>
       <c r="F12">
-        <v>21.742599999999999</v>
+        <v>21.8704</v>
       </c>
       <c r="G12">
-        <v>17.1004</v>
+        <v>16.715900000000001</v>
       </c>
       <c r="H12">
-        <v>14.563499999999999</v>
+        <v>14.096</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1275,22 +1275,22 @@
         <v>24</v>
       </c>
       <c r="C13">
-        <v>356.65199999999999</v>
+        <v>309.32299999999998</v>
       </c>
       <c r="D13">
-        <v>359.93099999999998</v>
+        <v>293.09500000000003</v>
       </c>
       <c r="E13">
-        <v>304.03899999999999</v>
+        <v>276.72699999999998</v>
       </c>
       <c r="F13">
-        <v>330.90800000000002</v>
+        <v>296.49200000000002</v>
       </c>
       <c r="G13">
-        <v>406.322</v>
+        <v>340.33499999999998</v>
       </c>
       <c r="H13">
-        <v>461.35500000000002</v>
+        <v>411.12299999999999</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1347,22 +1347,22 @@
         <v>15</v>
       </c>
       <c r="C16">
-        <v>0.140268</v>
+        <v>0.10978300000000001</v>
       </c>
       <c r="D16">
-        <v>0.142592</v>
+        <v>0.12669800000000001</v>
       </c>
       <c r="E16">
-        <v>0.36136800000000002</v>
+        <v>0.31293700000000002</v>
       </c>
       <c r="F16">
-        <v>0.129163</v>
+        <v>0.10714799999999999</v>
       </c>
       <c r="G16">
-        <v>0.41297499999999998</v>
+        <v>0.303929</v>
       </c>
       <c r="H16">
-        <v>0.39712900000000001</v>
+        <v>0.315056</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1399,22 +1399,22 @@
         <v>15</v>
       </c>
       <c r="C18">
-        <v>0.140268</v>
+        <v>0.10978300000000001</v>
       </c>
       <c r="D18">
-        <v>0.142592</v>
+        <v>0.12669800000000001</v>
       </c>
       <c r="E18">
-        <v>0.36136800000000002</v>
+        <v>0.31293700000000002</v>
       </c>
       <c r="F18">
-        <v>0.129163</v>
+        <v>0.10714799999999999</v>
       </c>
       <c r="G18">
-        <v>0.41297499999999998</v>
+        <v>0.303929</v>
       </c>
       <c r="H18">
-        <v>0.39712900000000001</v>
+        <v>0.315056</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1422,22 +1422,22 @@
         <v>30</v>
       </c>
       <c r="C19">
-        <v>23.988199999999999</v>
+        <v>19.6022</v>
       </c>
       <c r="D19">
-        <v>24.2728</v>
+        <v>19.402000000000001</v>
       </c>
       <c r="E19">
-        <v>17.868400000000001</v>
+        <v>16.054400000000001</v>
       </c>
       <c r="F19">
-        <v>22.5472</v>
+        <v>19.1982</v>
       </c>
       <c r="G19">
-        <v>18.574100000000001</v>
+        <v>14.821400000000001</v>
       </c>
       <c r="H19">
-        <v>18.742799999999999</v>
+        <v>15.788399999999999</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1445,22 +1445,22 @@
         <v>31</v>
       </c>
       <c r="C20">
-        <v>2.94503</v>
+        <v>2.94469</v>
       </c>
       <c r="D20">
-        <v>2.9447700000000001</v>
+        <v>2.9463300000000001</v>
       </c>
       <c r="E20">
-        <v>2.97038</v>
+        <v>2.96888</v>
       </c>
       <c r="F20">
-        <v>2.9411399999999999</v>
+        <v>2.9390800000000001</v>
       </c>
       <c r="G20">
-        <v>2.9695900000000002</v>
+        <v>2.9695100000000001</v>
       </c>
       <c r="H20">
-        <v>2.97193</v>
+        <v>2.9721600000000001</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1468,22 +1468,22 @@
         <v>32</v>
       </c>
       <c r="C21">
-        <v>2.4207200000000002</v>
+        <v>2.3419099999999999</v>
       </c>
       <c r="D21">
-        <v>2.4256099999999998</v>
+        <v>2.3389099999999998</v>
       </c>
       <c r="E21">
-        <v>2.2954300000000001</v>
+        <v>2.2541699999999998</v>
       </c>
       <c r="F21">
-        <v>2.3935399999999998</v>
+        <v>2.3317600000000001</v>
       </c>
       <c r="G21">
-        <v>2.3098000000000001</v>
+        <v>2.21698</v>
       </c>
       <c r="H21">
-        <v>2.3144</v>
+        <v>2.2467299999999999</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1491,22 +1491,22 @@
         <v>33</v>
       </c>
       <c r="C22">
-        <v>0.90210400000000002</v>
+        <v>0.92327199999999998</v>
       </c>
       <c r="D22">
-        <v>0.89769100000000002</v>
+        <v>0.924068</v>
       </c>
       <c r="E22">
-        <v>0.92332099999999995</v>
+        <v>0.91759299999999999</v>
       </c>
       <c r="F22">
-        <v>0.91858099999999998</v>
+        <v>0.92178199999999999</v>
       </c>
       <c r="G22">
-        <v>0.92507899999999998</v>
+        <v>0.91649199999999997</v>
       </c>
       <c r="H22">
-        <v>0.92573300000000003</v>
+        <v>0.91747199999999995</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1514,22 +1514,22 @@
         <v>34</v>
       </c>
       <c r="C23">
-        <v>0.91361099999999995</v>
+        <v>0.93115199999999998</v>
       </c>
       <c r="D23">
-        <v>0.90978999999999999</v>
+        <v>0.93179800000000002</v>
       </c>
       <c r="E23">
-        <v>0.93048799999999998</v>
+        <v>0.92461300000000002</v>
       </c>
       <c r="F23">
-        <v>0.92783499999999997</v>
+        <v>0.92973899999999998</v>
       </c>
       <c r="G23">
-        <v>0.932307</v>
+        <v>0.923122</v>
       </c>
       <c r="H23">
-        <v>0.93294900000000003</v>
+        <v>0.92441399999999996</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1537,22 +1537,22 @@
         <v>35</v>
       </c>
       <c r="C24">
-        <v>0.90210400000000002</v>
+        <v>0.92327199999999998</v>
       </c>
       <c r="D24">
-        <v>0.89769100000000002</v>
+        <v>0.924068</v>
       </c>
       <c r="E24">
-        <v>0.92332099999999995</v>
+        <v>0.91759299999999999</v>
       </c>
       <c r="F24">
-        <v>0.91858099999999998</v>
+        <v>0.92178199999999999</v>
       </c>
       <c r="G24">
-        <v>0.92507899999999998</v>
+        <v>0.91649199999999997</v>
       </c>
       <c r="H24">
-        <v>0.92573300000000003</v>
+        <v>0.91747199999999995</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1560,22 +1560,22 @@
         <v>36</v>
       </c>
       <c r="C25">
-        <v>0.91361099999999995</v>
+        <v>0.93115199999999998</v>
       </c>
       <c r="D25">
-        <v>0.90978999999999999</v>
+        <v>0.93179800000000002</v>
       </c>
       <c r="E25">
-        <v>0.93048799999999998</v>
+        <v>0.92461300000000002</v>
       </c>
       <c r="F25">
-        <v>0.92783499999999997</v>
+        <v>0.92973899999999998</v>
       </c>
       <c r="G25">
-        <v>0.932307</v>
+        <v>0.923122</v>
       </c>
       <c r="H25">
-        <v>0.93294900000000003</v>
+        <v>0.92441399999999996</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1583,22 +1583,22 @@
         <v>37</v>
       </c>
       <c r="C26">
-        <v>0.86803399999999997</v>
+        <v>0.87047300000000005</v>
       </c>
       <c r="D26">
-        <v>0.867367</v>
+        <v>0.87193100000000001</v>
       </c>
       <c r="E26">
-        <v>0.88047500000000001</v>
+        <v>0.88142699999999996</v>
       </c>
       <c r="F26">
-        <v>0.86838800000000005</v>
+        <v>0.86893399999999998</v>
       </c>
       <c r="G26">
-        <v>0.88016799999999995</v>
+        <v>0.88139299999999998</v>
       </c>
       <c r="H26">
-        <v>0.88013399999999997</v>
+        <v>0.88145600000000002</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1606,22 +1606,22 @@
         <v>38</v>
       </c>
       <c r="C27">
-        <v>0.90200599999999997</v>
+        <v>0.90299200000000002</v>
       </c>
       <c r="D27">
-        <v>0.90156099999999995</v>
+        <v>0.90400999999999998</v>
       </c>
       <c r="E27">
-        <v>0.90980700000000003</v>
+        <v>0.91014399999999995</v>
       </c>
       <c r="F27">
-        <v>0.90183899999999995</v>
+        <v>0.90163700000000002</v>
       </c>
       <c r="G27">
-        <v>0.90967399999999998</v>
+        <v>0.90976299999999999</v>
       </c>
       <c r="H27">
-        <v>0.90977300000000005</v>
+        <v>0.91015400000000002</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -1629,22 +1629,22 @@
         <v>39</v>
       </c>
       <c r="C28">
-        <v>0.85787000000000002</v>
+        <v>0.86814800000000003</v>
       </c>
       <c r="D28">
-        <v>0.85564600000000002</v>
+        <v>0.86967499999999998</v>
       </c>
       <c r="E28">
-        <v>0.876969</v>
+        <v>0.87651599999999996</v>
       </c>
       <c r="F28">
-        <v>0.86438899999999996</v>
+        <v>0.86652300000000004</v>
       </c>
       <c r="G28">
-        <v>0.87712999999999997</v>
+        <v>0.87657499999999999</v>
       </c>
       <c r="H28">
-        <v>0.87723499999999999</v>
+        <v>0.87656400000000001</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1652,22 +1652,22 @@
         <v>40</v>
       </c>
       <c r="C29">
-        <v>0.91875499999999999</v>
+        <v>0.90900499999999995</v>
       </c>
       <c r="D29">
-        <v>0.91913500000000004</v>
+        <v>0.91498800000000002</v>
       </c>
       <c r="E29">
-        <v>0.92350699999999997</v>
+        <v>0.92257199999999995</v>
       </c>
       <c r="F29">
-        <v>0.91383899999999996</v>
+        <v>0.90469599999999994</v>
       </c>
       <c r="G29">
-        <v>0.92390000000000005</v>
+        <v>0.92182900000000001</v>
       </c>
       <c r="H29">
-        <v>0.92379699999999998</v>
+        <v>0.92234700000000003</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1675,22 +1675,22 @@
         <v>41</v>
       </c>
       <c r="C30">
-        <v>0.90860099999999999</v>
+        <v>0.89763899999999996</v>
       </c>
       <c r="D30">
-        <v>0.90903699999999998</v>
+        <v>0.90433399999999997</v>
       </c>
       <c r="E30">
-        <v>0.91388599999999998</v>
+        <v>0.912748</v>
       </c>
       <c r="F30">
-        <v>0.90320199999999995</v>
+        <v>0.89297899999999997</v>
       </c>
       <c r="G30">
-        <v>0.91442699999999999</v>
+        <v>0.91187600000000002</v>
       </c>
       <c r="H30">
-        <v>0.91418699999999997</v>
+        <v>0.91243700000000005</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -1698,22 +1698,22 @@
         <v>42</v>
       </c>
       <c r="C31">
-        <v>0.92334799999999995</v>
+        <v>0.91330699999999998</v>
       </c>
       <c r="D31">
-        <v>0.92377900000000002</v>
+        <v>0.91910000000000003</v>
       </c>
       <c r="E31">
-        <v>0.92722499999999997</v>
+        <v>0.92589200000000005</v>
       </c>
       <c r="F31">
-        <v>0.91857599999999995</v>
+        <v>0.909165</v>
       </c>
       <c r="G31">
-        <v>0.92777500000000002</v>
+        <v>0.92486999999999997</v>
       </c>
       <c r="H31">
-        <v>0.92754800000000004</v>
+        <v>0.92547299999999999</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1721,22 +1721,22 @@
         <v>43</v>
       </c>
       <c r="C32">
-        <v>0.91954499999999995</v>
+        <v>0.90978999999999999</v>
       </c>
       <c r="D32">
-        <v>0.91935699999999998</v>
+        <v>0.913636</v>
       </c>
       <c r="E32">
-        <v>0.93476899999999996</v>
+        <v>0.92906699999999998</v>
       </c>
       <c r="F32">
-        <v>0.91680899999999999</v>
+        <v>0.90540299999999996</v>
       </c>
       <c r="G32">
-        <v>0.93612399999999996</v>
+        <v>0.92996100000000004</v>
       </c>
       <c r="H32">
-        <v>0.93630599999999997</v>
+        <v>0.92996199999999996</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -1744,22 +1744,22 @@
         <v>44</v>
       </c>
       <c r="C33">
-        <v>0.91113200000000005</v>
+        <v>0.90062799999999998</v>
       </c>
       <c r="D33">
-        <v>0.91091900000000003</v>
+        <v>0.90491100000000002</v>
       </c>
       <c r="E33">
-        <v>0.92834399999999995</v>
+        <v>0.92220599999999997</v>
       </c>
       <c r="F33">
-        <v>0.90831600000000001</v>
+        <v>0.896088</v>
       </c>
       <c r="G33">
-        <v>0.92978300000000003</v>
+        <v>0.923288</v>
       </c>
       <c r="H33">
-        <v>0.92994200000000005</v>
+        <v>0.92315800000000003</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -1767,22 +1767,22 @@
         <v>45</v>
       </c>
       <c r="C34">
-        <v>0.92512899999999998</v>
+        <v>0.91644199999999998</v>
       </c>
       <c r="D34">
-        <v>0.92523900000000003</v>
+        <v>0.92072799999999999</v>
       </c>
       <c r="E34">
-        <v>0.93347400000000003</v>
+        <v>0.93078799999999995</v>
       </c>
       <c r="F34">
-        <v>0.92147299999999999</v>
+        <v>0.912269</v>
       </c>
       <c r="G34">
-        <v>0.93412799999999996</v>
+        <v>0.93070399999999998</v>
       </c>
       <c r="H34">
-        <v>0.93425899999999995</v>
+        <v>0.93104699999999996</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -1822,7 +1822,7 @@
         <v>233.886</v>
       </c>
       <c r="D36">
-        <v>233.886</v>
+        <v>244.44200000000001</v>
       </c>
       <c r="E36">
         <v>294.67899999999997</v>
@@ -1848,7 +1848,7 @@
         <v>26.981300000000001</v>
       </c>
       <c r="D37">
-        <v>26.981300000000001</v>
+        <v>31.482900000000001</v>
       </c>
       <c r="E37">
         <v>96.662700000000001</v>
@@ -1874,7 +1874,7 @@
         <v>233.886</v>
       </c>
       <c r="D38">
-        <v>233.886</v>
+        <v>244.44200000000001</v>
       </c>
       <c r="E38">
         <v>294.67899999999997</v>
@@ -1900,7 +1900,7 @@
         <v>26.711500000000001</v>
       </c>
       <c r="D39">
-        <v>26.711500000000001</v>
+        <v>31.168099999999999</v>
       </c>
       <c r="E39">
         <v>95.695999999999998</v>
@@ -1949,22 +1949,22 @@
         <v>11</v>
       </c>
       <c r="C41">
-        <v>309.43299999999999</v>
+        <v>296.67899999999997</v>
       </c>
       <c r="D41">
-        <v>310.40300000000002</v>
+        <v>309.03399999999999</v>
       </c>
       <c r="E41">
-        <v>365.38</v>
+        <v>358.50299999999999</v>
       </c>
       <c r="F41">
-        <v>318.81700000000001</v>
+        <v>309.13900000000001</v>
       </c>
       <c r="G41">
-        <v>372.096</v>
+        <v>357.572</v>
       </c>
       <c r="H41">
-        <v>360.33199999999999</v>
+        <v>349.49799999999999</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -1975,22 +1975,22 @@
         <v>47</v>
       </c>
       <c r="C42">
-        <v>65.325299999999999</v>
+        <v>57.921599999999998</v>
       </c>
       <c r="D42">
-        <v>65.735600000000005</v>
+        <v>66.9191</v>
       </c>
       <c r="E42">
-        <v>193.179</v>
+        <v>180.816</v>
       </c>
       <c r="F42">
-        <v>60.910299999999999</v>
+        <v>55.176000000000002</v>
       </c>
       <c r="G42">
-        <v>213.34299999999999</v>
+        <v>186.17</v>
       </c>
       <c r="H42">
-        <v>208.52500000000001</v>
+        <v>187.59</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -2001,22 +2001,22 @@
         <v>11</v>
       </c>
       <c r="C43">
-        <v>309.43299999999999</v>
+        <v>296.67899999999997</v>
       </c>
       <c r="D43">
-        <v>310.40300000000002</v>
+        <v>309.03399999999999</v>
       </c>
       <c r="E43">
-        <v>365.38</v>
+        <v>358.50299999999999</v>
       </c>
       <c r="F43">
-        <v>318.81700000000001</v>
+        <v>309.13900000000001</v>
       </c>
       <c r="G43">
-        <v>372.096</v>
+        <v>357.572</v>
       </c>
       <c r="H43">
-        <v>360.33199999999999</v>
+        <v>349.49799999999999</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2027,22 +2027,22 @@
         <v>47</v>
       </c>
       <c r="C44">
-        <v>65.325299999999999</v>
+        <v>57.921599999999998</v>
       </c>
       <c r="D44">
-        <v>65.735600000000005</v>
+        <v>66.9191</v>
       </c>
       <c r="E44">
-        <v>193.179</v>
+        <v>180.816</v>
       </c>
       <c r="F44">
-        <v>60.910299999999999</v>
+        <v>55.176000000000002</v>
       </c>
       <c r="G44">
-        <v>213.34299999999999</v>
+        <v>186.17</v>
       </c>
       <c r="H44">
-        <v>208.52500000000001</v>
+        <v>187.59</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2053,22 +2053,22 @@
         <v>47</v>
       </c>
       <c r="C45">
-        <v>63.990299999999998</v>
+        <v>56.648899999999998</v>
       </c>
       <c r="D45">
-        <v>64.400199999999998</v>
+        <v>65.442400000000006</v>
       </c>
       <c r="E45">
-        <v>188.79599999999999</v>
+        <v>176.55500000000001</v>
       </c>
       <c r="F45">
-        <v>59.6389</v>
+        <v>53.964599999999997</v>
       </c>
       <c r="G45">
-        <v>208.577</v>
+        <v>181.649</v>
       </c>
       <c r="H45">
-        <v>203.86099999999999</v>
+        <v>183.12799999999999</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -2079,22 +2079,22 @@
         <v>47</v>
       </c>
       <c r="C46">
-        <v>65.325299999999999</v>
+        <v>57.921599999999998</v>
       </c>
       <c r="D46">
-        <v>65.735600000000005</v>
+        <v>66.9191</v>
       </c>
       <c r="E46">
-        <v>193.179</v>
+        <v>180.816</v>
       </c>
       <c r="F46">
-        <v>60.910299999999999</v>
+        <v>55.176000000000002</v>
       </c>
       <c r="G46">
-        <v>213.34299999999999</v>
+        <v>186.17</v>
       </c>
       <c r="H46">
-        <v>208.52500000000001</v>
+        <v>187.59</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2105,22 +2105,22 @@
         <v>47</v>
       </c>
       <c r="C47">
-        <v>55.419199999999996</v>
+        <v>50.479199999999999</v>
       </c>
       <c r="D47">
-        <v>55.665100000000002</v>
+        <v>58.136099999999999</v>
       </c>
       <c r="E47">
-        <v>166.953</v>
+        <v>157.97</v>
       </c>
       <c r="F47">
-        <v>52.266500000000001</v>
+        <v>48.3003</v>
       </c>
       <c r="G47">
-        <v>183.58600000000001</v>
+        <v>163.95599999999999</v>
       </c>
       <c r="H47">
-        <v>179.27199999999999</v>
+        <v>164.13</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2131,22 +2131,22 @@
         <v>11</v>
       </c>
       <c r="C48">
-        <v>629.21900000000005</v>
+        <v>589.36300000000006</v>
       </c>
       <c r="D48">
-        <v>632.35199999999998</v>
+        <v>612.31100000000004</v>
       </c>
       <c r="E48">
-        <v>710.14599999999996</v>
+        <v>689.09900000000005</v>
       </c>
       <c r="F48">
-        <v>641.58900000000006</v>
+        <v>611.73800000000006</v>
       </c>
       <c r="G48">
-        <v>725.35</v>
+        <v>680.65800000000002</v>
       </c>
       <c r="H48">
-        <v>704.81799999999998</v>
+        <v>671.39099999999996</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2157,22 +2157,22 @@
         <v>47</v>
       </c>
       <c r="C49">
-        <v>640.75900000000001</v>
+        <v>523.60199999999998</v>
       </c>
       <c r="D49">
-        <v>648.36199999999997</v>
+        <v>604.72199999999998</v>
       </c>
       <c r="E49">
-        <v>1709.93</v>
+        <v>1536.34</v>
       </c>
       <c r="F49">
-        <v>579.76800000000003</v>
+        <v>493.65300000000002</v>
       </c>
       <c r="G49">
-        <v>1915.89</v>
+        <v>1528.81</v>
       </c>
       <c r="H49">
-        <v>1880.12</v>
+        <v>1583.76</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2183,22 +2183,22 @@
         <v>47</v>
       </c>
       <c r="C50">
-        <v>623.41</v>
+        <v>509.37599999999998</v>
       </c>
       <c r="D50">
-        <v>630.82500000000005</v>
+        <v>588.02</v>
       </c>
       <c r="E50">
-        <v>1660.19</v>
+        <v>1491.15</v>
       </c>
       <c r="F50">
-        <v>564.13800000000003</v>
+        <v>480.36099999999999</v>
       </c>
       <c r="G50">
-        <v>1860.37</v>
+        <v>1483.38</v>
       </c>
       <c r="H50">
-        <v>1825.61</v>
+        <v>1537.01</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2209,22 +2209,22 @@
         <v>47</v>
       </c>
       <c r="C51">
-        <v>608.58799999999997</v>
+        <v>497.22199999999998</v>
       </c>
       <c r="D51">
-        <v>615.84199999999998</v>
+        <v>573.76800000000003</v>
       </c>
       <c r="E51">
-        <v>1617.92</v>
+        <v>1452.78</v>
       </c>
       <c r="F51">
-        <v>550.78099999999995</v>
+        <v>468.99900000000002</v>
       </c>
       <c r="G51">
-        <v>1813.17</v>
+        <v>1444.83</v>
       </c>
       <c r="H51">
-        <v>1779.29</v>
+        <v>1497.32</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -2235,22 +2235,22 @@
         <v>11</v>
       </c>
       <c r="C52">
-        <v>1566.55</v>
+        <v>1467.32</v>
       </c>
       <c r="D52">
-        <v>1575.58</v>
+        <v>1497.91</v>
       </c>
       <c r="E52">
-        <v>1630.98</v>
+        <v>1568.7</v>
       </c>
       <c r="F52">
-        <v>1599.96</v>
+        <v>1531.4</v>
       </c>
       <c r="G52">
-        <v>1669.45</v>
+        <v>1534.86</v>
       </c>
       <c r="H52">
-        <v>1624.79</v>
+        <v>1525.09</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -2261,22 +2261,22 @@
         <v>11</v>
       </c>
       <c r="C53">
-        <v>1448.94</v>
+        <v>1356.64</v>
       </c>
       <c r="D53">
-        <v>1457.28</v>
+        <v>1386.22</v>
       </c>
       <c r="E53">
-        <v>1514.87</v>
+        <v>1457.32</v>
       </c>
       <c r="F53">
-        <v>1479.91</v>
+        <v>1415.96</v>
       </c>
       <c r="G53">
-        <v>1550.59</v>
+        <v>1426.47</v>
       </c>
       <c r="H53">
-        <v>1508.8</v>
+        <v>1416.81</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -2287,22 +2287,22 @@
         <v>11</v>
       </c>
       <c r="C54">
-        <v>1448.94</v>
+        <v>1356.64</v>
       </c>
       <c r="D54">
-        <v>1457.28</v>
+        <v>1386.22</v>
       </c>
       <c r="E54">
-        <v>1514.87</v>
+        <v>1457.32</v>
       </c>
       <c r="F54">
-        <v>1479.91</v>
+        <v>1415.96</v>
       </c>
       <c r="G54">
-        <v>1550.59</v>
+        <v>1426.47</v>
       </c>
       <c r="H54">
-        <v>1508.8</v>
+        <v>1416.81</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -2313,22 +2313,22 @@
         <v>47</v>
       </c>
       <c r="C55">
-        <v>206.649</v>
+        <v>168.85400000000001</v>
       </c>
       <c r="D55">
-        <v>209.131</v>
+        <v>194.74</v>
       </c>
       <c r="E55">
-        <v>544.68499999999995</v>
+        <v>489.334</v>
       </c>
       <c r="F55">
-        <v>187.268</v>
+        <v>159.57300000000001</v>
       </c>
       <c r="G55">
-        <v>610.58000000000004</v>
+        <v>486.55399999999997</v>
       </c>
       <c r="H55">
-        <v>598.697</v>
+        <v>503.78100000000001</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -2339,22 +2339,22 @@
         <v>47</v>
       </c>
       <c r="C56">
-        <v>206.649</v>
+        <v>168.85400000000001</v>
       </c>
       <c r="D56">
-        <v>209.131</v>
+        <v>194.74</v>
       </c>
       <c r="E56">
-        <v>544.68499999999995</v>
+        <v>489.334</v>
       </c>
       <c r="F56">
-        <v>187.268</v>
+        <v>159.57300000000001</v>
       </c>
       <c r="G56">
-        <v>610.58000000000004</v>
+        <v>486.55399999999997</v>
       </c>
       <c r="H56">
-        <v>598.697</v>
+        <v>503.78100000000001</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -2365,22 +2365,22 @@
         <v>11</v>
       </c>
       <c r="C57">
-        <v>1143.51</v>
+        <v>1070.3699999999999</v>
       </c>
       <c r="D57">
-        <v>1150.3</v>
+        <v>1092.93</v>
       </c>
       <c r="E57">
-        <v>1194.58</v>
+        <v>1147.48</v>
       </c>
       <c r="F57">
-        <v>1171.05</v>
+        <v>1121.21</v>
       </c>
       <c r="G57">
-        <v>1223.98</v>
+        <v>1122.32</v>
       </c>
       <c r="H57">
-        <v>1189.28</v>
+        <v>1113.97</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -2391,22 +2391,22 @@
         <v>11</v>
       </c>
       <c r="C58">
-        <v>941.58100000000002</v>
+        <v>887.49099999999999</v>
       </c>
       <c r="D58">
-        <v>947.03599999999994</v>
+        <v>906.29700000000003</v>
       </c>
       <c r="E58">
-        <v>993.36099999999999</v>
+        <v>957.60599999999999</v>
       </c>
       <c r="F58">
-        <v>968.29100000000005</v>
+        <v>933.11300000000006</v>
       </c>
       <c r="G58">
-        <v>1017.11</v>
+        <v>939.01900000000001</v>
       </c>
       <c r="H58">
-        <v>986.59900000000005</v>
+        <v>928.97699999999998</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -2417,22 +2417,22 @@
         <v>47</v>
       </c>
       <c r="C59">
-        <v>85.366699999999994</v>
+        <v>72.100899999999996</v>
       </c>
       <c r="D59">
-        <v>86.2179</v>
+        <v>83.260999999999996</v>
       </c>
       <c r="E59">
-        <v>237.291</v>
+        <v>217.07900000000001</v>
       </c>
       <c r="F59">
-        <v>78.238699999999994</v>
+        <v>68.434899999999999</v>
       </c>
       <c r="G59">
-        <v>264.34300000000002</v>
+        <v>219.46700000000001</v>
       </c>
       <c r="H59">
-        <v>258.68299999999999</v>
+        <v>224.22800000000001</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -2443,22 +2443,22 @@
         <v>11</v>
       </c>
       <c r="C60">
-        <v>526.10299999999995</v>
+        <v>484.173</v>
       </c>
       <c r="D60">
-        <v>529.76</v>
+        <v>500.01900000000001</v>
       </c>
       <c r="E60">
-        <v>567.94500000000005</v>
+        <v>544.62</v>
       </c>
       <c r="F60">
-        <v>536.53800000000001</v>
+        <v>506.63499999999999</v>
       </c>
       <c r="G60">
-        <v>583.47500000000002</v>
+        <v>532.947</v>
       </c>
       <c r="H60">
-        <v>565.09299999999996</v>
+        <v>527.87400000000002</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
@@ -2469,22 +2469,22 @@
         <v>47</v>
       </c>
       <c r="C61">
-        <v>69.3523</v>
+        <v>60.354100000000003</v>
       </c>
       <c r="D61">
-        <v>69.887200000000007</v>
+        <v>69.727999999999994</v>
       </c>
       <c r="E61">
-        <v>200.45500000000001</v>
+        <v>186.042</v>
       </c>
       <c r="F61">
-        <v>64.207400000000007</v>
+        <v>57.410400000000003</v>
       </c>
       <c r="G61">
-        <v>222.09200000000001</v>
+        <v>190.29599999999999</v>
       </c>
       <c r="H61">
-        <v>217.179</v>
+        <v>192.714</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -2495,22 +2495,22 @@
         <v>11</v>
       </c>
       <c r="C62">
-        <v>526.10299999999995</v>
+        <v>484.173</v>
       </c>
       <c r="D62">
-        <v>529.76</v>
+        <v>500.01900000000001</v>
       </c>
       <c r="E62">
-        <v>567.94500000000005</v>
+        <v>544.62</v>
       </c>
       <c r="F62">
-        <v>536.53800000000001</v>
+        <v>506.63499999999999</v>
       </c>
       <c r="G62">
-        <v>583.47500000000002</v>
+        <v>532.947</v>
       </c>
       <c r="H62">
-        <v>565.09299999999996</v>
+        <v>527.87400000000002</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -2521,22 +2521,22 @@
         <v>11</v>
       </c>
       <c r="C63">
-        <v>526.10299999999995</v>
+        <v>484.173</v>
       </c>
       <c r="D63">
-        <v>529.76</v>
+        <v>500.01799999999997</v>
       </c>
       <c r="E63">
-        <v>567.94399999999996</v>
+        <v>544.62</v>
       </c>
       <c r="F63">
-        <v>536.53700000000003</v>
+        <v>506.63499999999999</v>
       </c>
       <c r="G63">
-        <v>583.47500000000002</v>
+        <v>532.947</v>
       </c>
       <c r="H63">
-        <v>565.09299999999996</v>
+        <v>527.87400000000002</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
@@ -2547,22 +2547,22 @@
         <v>47</v>
       </c>
       <c r="C64">
-        <v>69.3523</v>
+        <v>60.354100000000003</v>
       </c>
       <c r="D64">
-        <v>69.887200000000007</v>
+        <v>69.727999999999994</v>
       </c>
       <c r="E64">
-        <v>200.45500000000001</v>
+        <v>186.042</v>
       </c>
       <c r="F64">
-        <v>64.207400000000007</v>
+        <v>57.410400000000003</v>
       </c>
       <c r="G64">
-        <v>222.09200000000001</v>
+        <v>190.29599999999999</v>
       </c>
       <c r="H64">
-        <v>217.179</v>
+        <v>192.714</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
@@ -2654,7 +2654,7 @@
         <v>1</v>
       </c>
       <c r="G68">
-        <v>1</v>
+        <v>0.99653099999999994</v>
       </c>
       <c r="H68">
         <v>1</v>
@@ -2665,22 +2665,22 @@
         <v>82</v>
       </c>
       <c r="C69">
-        <v>3.3588800000000001</v>
+        <v>2.9230800000000001</v>
       </c>
       <c r="D69">
-        <v>3.3847800000000001</v>
+        <v>3.3770799999999999</v>
       </c>
       <c r="E69">
-        <v>2.8767200000000002</v>
+        <v>2.66988</v>
       </c>
       <c r="F69">
-        <v>3.7693699999999999</v>
+        <v>3.3703400000000001</v>
       </c>
       <c r="G69">
-        <v>2.1918700000000002</v>
+        <v>1.87808</v>
       </c>
       <c r="H69">
-        <v>2.1433900000000001</v>
+        <v>1.90194</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2691,22 +2691,22 @@
         <v>15</v>
       </c>
       <c r="C70">
-        <v>19.5746</v>
+        <v>17.781600000000001</v>
       </c>
       <c r="D70">
-        <v>19.653500000000001</v>
+        <v>20.2135</v>
       </c>
       <c r="E70">
-        <v>54.414200000000001</v>
+        <v>51.634900000000002</v>
       </c>
       <c r="F70">
-        <v>17.952300000000001</v>
+        <v>16.523900000000001</v>
       </c>
       <c r="G70">
-        <v>59.435600000000001</v>
+        <v>53.423999999999999</v>
       </c>
       <c r="H70">
-        <v>59.105600000000003</v>
+        <v>54.365200000000002</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -2717,22 +2717,22 @@
         <v>15</v>
       </c>
       <c r="C71">
-        <v>66.896600000000007</v>
+        <v>60.768900000000002</v>
       </c>
       <c r="D71">
-        <v>67.166200000000003</v>
+        <v>60.523800000000001</v>
       </c>
       <c r="E71">
-        <v>58.264000000000003</v>
+        <v>55.2881</v>
       </c>
       <c r="F71">
-        <v>65.156099999999995</v>
+        <v>59.971800000000002</v>
       </c>
       <c r="G71">
-        <v>59.376100000000001</v>
+        <v>53.3705</v>
       </c>
       <c r="H71">
-        <v>59.7027</v>
+        <v>54.914400000000001</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -2743,22 +2743,22 @@
         <v>15</v>
       </c>
       <c r="C72">
-        <v>6.4179700000000004</v>
+        <v>5.42835</v>
       </c>
       <c r="D72">
-        <v>6.4746800000000002</v>
+        <v>6.1997299999999997</v>
       </c>
       <c r="E72">
-        <v>16.690000000000001</v>
+        <v>15.3047</v>
       </c>
       <c r="F72">
-        <v>5.7383899999999999</v>
+        <v>5.0006300000000001</v>
       </c>
       <c r="G72">
-        <v>18.470099999999999</v>
+        <v>15.4002</v>
       </c>
       <c r="H72">
-        <v>18.389700000000001</v>
+        <v>16.0122</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2769,22 +2769,22 @@
         <v>15</v>
       </c>
       <c r="C73">
-        <v>21.933599999999998</v>
+        <v>18.551500000000001</v>
       </c>
       <c r="D73">
-        <v>22.127400000000002</v>
+        <v>18.563400000000001</v>
       </c>
       <c r="E73">
-        <v>17.870899999999999</v>
+        <v>16.387499999999999</v>
       </c>
       <c r="F73">
-        <v>20.826899999999998</v>
+        <v>18.1493</v>
       </c>
       <c r="G73">
-        <v>18.451599999999999</v>
+        <v>15.3848</v>
       </c>
       <c r="H73">
-        <v>18.575500000000002</v>
+        <v>16.173999999999999</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -2795,22 +2795,22 @@
         <v>15</v>
       </c>
       <c r="C74">
-        <v>13.156599999999999</v>
+        <v>12.353199999999999</v>
       </c>
       <c r="D74">
-        <v>13.178800000000001</v>
+        <v>14.0137</v>
       </c>
       <c r="E74">
-        <v>37.7241</v>
+        <v>36.330199999999998</v>
       </c>
       <c r="F74">
-        <v>12.213900000000001</v>
+        <v>11.523300000000001</v>
       </c>
       <c r="G74">
-        <v>40.965600000000002</v>
+        <v>38.023800000000001</v>
       </c>
       <c r="H74">
-        <v>40.715899999999998</v>
+        <v>38.353000000000002</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2821,22 +2821,22 @@
         <v>15</v>
       </c>
       <c r="C75">
-        <v>44.963000000000001</v>
+        <v>42.217399999999998</v>
       </c>
       <c r="D75">
-        <v>45.038899999999998</v>
+        <v>41.9604</v>
       </c>
       <c r="E75">
-        <v>40.393099999999997</v>
+        <v>38.900599999999997</v>
       </c>
       <c r="F75">
-        <v>44.3292</v>
+        <v>41.822600000000001</v>
       </c>
       <c r="G75">
-        <v>40.924599999999998</v>
+        <v>37.985700000000001</v>
       </c>
       <c r="H75">
-        <v>41.127200000000002</v>
+        <v>38.740400000000001</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -2847,22 +2847,22 @@
         <v>15</v>
       </c>
       <c r="C76">
-        <v>6.4180700000000002</v>
+        <v>5.4283799999999998</v>
       </c>
       <c r="D76">
-        <v>6.4747199999999996</v>
+        <v>6.1997200000000001</v>
       </c>
       <c r="E76">
-        <v>16.690100000000001</v>
+        <v>15.305</v>
       </c>
       <c r="F76">
-        <v>5.7387899999999998</v>
+        <v>5.0014399999999997</v>
       </c>
       <c r="G76">
-        <v>18.470099999999999</v>
+        <v>15.4002</v>
       </c>
       <c r="H76">
-        <v>18.389700000000001</v>
+        <v>16.0122</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -2873,22 +2873,22 @@
         <v>15</v>
       </c>
       <c r="C77">
-        <v>10.3161</v>
+        <v>9.6356400000000004</v>
       </c>
       <c r="D77">
-        <v>10.3584</v>
+        <v>9.7214899999999993</v>
       </c>
       <c r="E77">
-        <v>9.8577899999999996</v>
+        <v>9.5664599999999993</v>
       </c>
       <c r="F77">
-        <v>10.041700000000001</v>
+        <v>9.5132700000000003</v>
       </c>
       <c r="G77">
-        <v>9.9684299999999997</v>
+        <v>9.3369400000000002</v>
       </c>
       <c r="H77">
-        <v>9.99254</v>
+        <v>9.52515</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -2899,22 +2899,22 @@
         <v>15</v>
       </c>
       <c r="C78">
-        <v>6.4180700000000002</v>
+        <v>5.4283799999999998</v>
       </c>
       <c r="D78">
-        <v>6.4747199999999996</v>
+        <v>6.1997200000000001</v>
       </c>
       <c r="E78">
-        <v>16.690100000000001</v>
+        <v>15.305</v>
       </c>
       <c r="F78">
-        <v>5.7387899999999998</v>
+        <v>5.0014399999999997</v>
       </c>
       <c r="G78">
-        <v>18.470099999999999</v>
+        <v>15.4002</v>
       </c>
       <c r="H78">
-        <v>18.389700000000001</v>
+        <v>16.0122</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -2925,22 +2925,22 @@
         <v>15</v>
       </c>
       <c r="C79">
-        <v>1.4997499999999999</v>
+        <v>1.50234</v>
       </c>
       <c r="D79">
-        <v>1.4989600000000001</v>
+        <v>1.5142899999999999</v>
       </c>
       <c r="E79">
-        <v>1.5526</v>
+        <v>1.56097</v>
       </c>
       <c r="F79">
-        <v>1.4965900000000001</v>
+        <v>1.49577</v>
       </c>
       <c r="G79">
-        <v>1.5498099999999999</v>
+        <v>1.5687199999999999</v>
       </c>
       <c r="H79">
-        <v>1.55002</v>
+        <v>1.5637099999999999</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -2951,22 +2951,22 @@
         <v>15</v>
       </c>
       <c r="C80">
-        <v>5.2105499999999996</v>
+        <v>4.3982000000000001</v>
       </c>
       <c r="D80">
-        <v>5.2576200000000002</v>
+        <v>5.0244799999999996</v>
       </c>
       <c r="E80">
-        <v>13.5465</v>
+        <v>12.4039</v>
       </c>
       <c r="F80">
-        <v>4.6628100000000003</v>
+        <v>4.0582900000000004</v>
       </c>
       <c r="G80">
-        <v>15.0044</v>
+        <v>12.4701</v>
       </c>
       <c r="H80">
-        <v>14.925000000000001</v>
+        <v>12.964700000000001</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
@@ -2977,22 +2977,22 @@
         <v>15</v>
       </c>
       <c r="C81">
-        <v>6.0449000000000002</v>
+        <v>5.1038899999999998</v>
       </c>
       <c r="D81">
-        <v>6.0993399999999998</v>
+        <v>5.8304400000000003</v>
       </c>
       <c r="E81">
-        <v>15.716200000000001</v>
+        <v>14.3935</v>
       </c>
       <c r="F81">
-        <v>5.4088500000000002</v>
+        <v>4.7084799999999998</v>
       </c>
       <c r="G81">
-        <v>17.4055</v>
+        <v>14.472099999999999</v>
       </c>
       <c r="H81">
-        <v>17.3157</v>
+        <v>15.0463</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
@@ -3003,22 +3003,22 @@
         <v>15</v>
       </c>
       <c r="C82">
-        <v>2.2568100000000002</v>
+        <v>2.2567699999999999</v>
       </c>
       <c r="D82">
-        <v>2.25678</v>
+        <v>2.2583199999999999</v>
       </c>
       <c r="E82">
-        <v>2.2567499999999998</v>
+        <v>2.2576200000000002</v>
       </c>
       <c r="F82">
-        <v>2.25501</v>
+        <v>2.2549600000000001</v>
       </c>
       <c r="G82">
-        <v>2.2563200000000001</v>
+        <v>2.2581500000000001</v>
       </c>
       <c r="H82">
-        <v>2.2563900000000001</v>
+        <v>2.2577500000000001</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -3029,22 +3029,22 @@
         <v>15</v>
       </c>
       <c r="C83">
-        <v>6.17326</v>
+        <v>5.2124600000000001</v>
       </c>
       <c r="D83">
-        <v>6.2288300000000003</v>
+        <v>5.95444</v>
       </c>
       <c r="E83">
-        <v>16.05</v>
+        <v>14.6996</v>
       </c>
       <c r="F83">
-        <v>5.5236299999999998</v>
+        <v>4.8085000000000004</v>
       </c>
       <c r="G83">
-        <v>17.774899999999999</v>
+        <v>14.780099999999999</v>
       </c>
       <c r="H83">
-        <v>17.683499999999999</v>
+        <v>15.3666</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -3055,22 +3055,22 @@
         <v>15</v>
       </c>
       <c r="C84">
-        <v>6.0298499999999997</v>
+        <v>6.0284300000000002</v>
       </c>
       <c r="D84">
-        <v>6.0297499999999999</v>
+        <v>6.0337500000000004</v>
       </c>
       <c r="E84">
-        <v>6.0791599999999999</v>
+        <v>6.0740699999999999</v>
       </c>
       <c r="F84">
-        <v>6.0249699999999997</v>
+        <v>6.0228000000000002</v>
       </c>
       <c r="G84">
-        <v>6.0793400000000002</v>
+        <v>6.0744999999999996</v>
       </c>
       <c r="H84">
-        <v>6.0800299999999998</v>
+        <v>6.0768300000000002</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
@@ -3081,22 +3081,22 @@
         <v>15</v>
       </c>
       <c r="C85">
-        <v>6.17326</v>
+        <v>5.2124600000000001</v>
       </c>
       <c r="D85">
-        <v>6.2288300000000003</v>
+        <v>5.95444</v>
       </c>
       <c r="E85">
-        <v>16.05</v>
+        <v>14.6996</v>
       </c>
       <c r="F85">
-        <v>5.5236299999999998</v>
+        <v>4.8085000000000004</v>
       </c>
       <c r="G85">
-        <v>17.774899999999999</v>
+        <v>14.780099999999999</v>
       </c>
       <c r="H85">
-        <v>17.683499999999999</v>
+        <v>15.3666</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -3107,22 +3107,22 @@
         <v>15</v>
       </c>
       <c r="C86">
-        <v>13.245200000000001</v>
+        <v>12.855499999999999</v>
       </c>
       <c r="D86">
-        <v>13.270799999999999</v>
+        <v>12.851100000000001</v>
       </c>
       <c r="E86">
-        <v>12.7249</v>
+        <v>12.507999999999999</v>
       </c>
       <c r="F86">
-        <v>13.113200000000001</v>
+        <v>12.8116</v>
       </c>
       <c r="G86">
-        <v>12.8005</v>
+        <v>12.318300000000001</v>
       </c>
       <c r="H86">
-        <v>12.816599999999999</v>
+        <v>12.4679</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
@@ -3133,22 +3133,22 @@
         <v>15</v>
       </c>
       <c r="C87">
-        <v>6.4941599999999999</v>
+        <v>5.4838800000000001</v>
       </c>
       <c r="D87">
-        <v>6.5525700000000002</v>
+        <v>6.2644200000000003</v>
       </c>
       <c r="E87">
-        <v>16.884499999999999</v>
+        <v>15.4649</v>
       </c>
       <c r="F87">
-        <v>5.8105700000000002</v>
+        <v>5.0585800000000001</v>
       </c>
       <c r="G87">
-        <v>18.698399999999999</v>
+        <v>15.5501</v>
       </c>
       <c r="H87">
-        <v>18.603000000000002</v>
+        <v>16.167200000000001</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
@@ -3159,22 +3159,22 @@
         <v>15</v>
       </c>
       <c r="C88">
-        <v>13.156599999999999</v>
+        <v>12.353199999999999</v>
       </c>
       <c r="D88">
-        <v>13.178800000000001</v>
+        <v>14.0137</v>
       </c>
       <c r="E88">
-        <v>37.7241</v>
+        <v>36.330199999999998</v>
       </c>
       <c r="F88">
-        <v>12.213900000000001</v>
+        <v>11.523300000000001</v>
       </c>
       <c r="G88">
-        <v>40.965600000000002</v>
+        <v>38.023800000000001</v>
       </c>
       <c r="H88">
-        <v>40.715899999999998</v>
+        <v>38.353000000000002</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -3185,22 +3185,22 @@
         <v>15</v>
       </c>
       <c r="C89">
-        <v>19.6508</v>
+        <v>17.8371</v>
       </c>
       <c r="D89">
-        <v>19.731400000000001</v>
+        <v>20.278199999999998</v>
       </c>
       <c r="E89">
-        <v>54.608699999999999</v>
+        <v>51.795099999999998</v>
       </c>
       <c r="F89">
-        <v>18.0245</v>
+        <v>16.581800000000001</v>
       </c>
       <c r="G89">
-        <v>59.663899999999998</v>
+        <v>53.573900000000002</v>
       </c>
       <c r="H89">
-        <v>59.318899999999999</v>
+        <v>54.520200000000003</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
@@ -3211,22 +3211,22 @@
         <v>15</v>
       </c>
       <c r="C90">
-        <v>19.6508</v>
+        <v>17.8371</v>
       </c>
       <c r="D90">
-        <v>19.731400000000001</v>
+        <v>20.278199999999998</v>
       </c>
       <c r="E90">
-        <v>54.608699999999999</v>
+        <v>51.795099999999998</v>
       </c>
       <c r="F90">
-        <v>18.0245</v>
+        <v>16.581800000000001</v>
       </c>
       <c r="G90">
-        <v>59.663899999999998</v>
+        <v>53.573900000000002</v>
       </c>
       <c r="H90">
-        <v>59.318899999999999</v>
+        <v>54.520200000000003</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
@@ -3237,22 +3237,22 @@
         <v>15</v>
       </c>
       <c r="C91">
-        <v>38.793700000000001</v>
+        <v>38.8172</v>
       </c>
       <c r="D91">
-        <v>38.788800000000002</v>
+        <v>38.816899999999997</v>
       </c>
       <c r="E91">
-        <v>38.753</v>
+        <v>38.7821</v>
       </c>
       <c r="F91">
-        <v>38.813600000000001</v>
+        <v>38.805799999999998</v>
       </c>
       <c r="G91">
-        <v>38.734400000000001</v>
+        <v>38.794600000000003</v>
       </c>
       <c r="H91">
-        <v>38.756300000000003</v>
+        <v>38.798699999999997</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
@@ -3260,22 +3260,22 @@
         <v>105</v>
       </c>
       <c r="C92">
-        <v>108.54900000000001</v>
+        <v>150.81200000000001</v>
       </c>
       <c r="D92">
-        <v>106.093</v>
+        <v>123.117</v>
       </c>
       <c r="E92">
-        <v>36.8309</v>
+        <v>43.928100000000001</v>
       </c>
       <c r="F92">
-        <v>111.51300000000001</v>
+        <v>143.38800000000001</v>
       </c>
       <c r="G92">
-        <v>31.572299999999998</v>
+        <v>45.866599999999998</v>
       </c>
       <c r="H92">
-        <v>34.823399999999999</v>
+        <v>46.156100000000002</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
@@ -3283,22 +3283,22 @@
         <v>106</v>
       </c>
       <c r="C93">
-        <v>0.98859799999999998</v>
+        <v>0.98070299999999999</v>
       </c>
       <c r="D93">
-        <v>0.98900699999999997</v>
+        <v>0.98605200000000004</v>
       </c>
       <c r="E93">
-        <v>0.997977</v>
+        <v>0.99731800000000004</v>
       </c>
       <c r="F93">
-        <v>0.98809499999999995</v>
+        <v>0.98219999999999996</v>
       </c>
       <c r="G93">
-        <v>0.99841899999999995</v>
+        <v>0.99712699999999999</v>
       </c>
       <c r="H93">
-        <v>0.99815100000000001</v>
+        <v>0.99709800000000004</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
@@ -3306,22 +3306,22 @@
         <v>107</v>
       </c>
       <c r="C94">
-        <v>0.22132399999999999</v>
+        <v>0.16630600000000001</v>
       </c>
       <c r="D94">
-        <v>0.22598299999999999</v>
+        <v>0.198243</v>
       </c>
       <c r="E94">
-        <v>0.49698599999999998</v>
+        <v>0.42729299999999998</v>
       </c>
       <c r="F94">
-        <v>0.22661500000000001</v>
+        <v>0.18224899999999999</v>
       </c>
       <c r="G94">
-        <v>0.56243100000000001</v>
+        <v>0.408331</v>
       </c>
       <c r="H94">
-        <v>0.50225500000000001</v>
+        <v>0.39486100000000002</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
@@ -3332,22 +3332,22 @@
         <v>109</v>
       </c>
       <c r="C95">
-        <v>75.841399999999993</v>
+        <v>62.997</v>
       </c>
       <c r="D95">
-        <v>76.819800000000001</v>
+        <v>64.848200000000006</v>
       </c>
       <c r="E95">
-        <v>71.273600000000002</v>
+        <v>64.337400000000002</v>
       </c>
       <c r="F95">
-        <v>74.714399999999998</v>
+        <v>64.954499999999996</v>
       </c>
       <c r="G95">
-        <v>74.696700000000007</v>
+        <v>60.048699999999997</v>
       </c>
       <c r="H95">
-        <v>72.732699999999994</v>
+        <v>61.807400000000001</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
@@ -3358,22 +3358,22 @@
         <v>109</v>
       </c>
       <c r="C96">
-        <v>75.841399999999993</v>
+        <v>62.997</v>
       </c>
       <c r="D96">
-        <v>76.819800000000001</v>
+        <v>64.848200000000006</v>
       </c>
       <c r="E96">
-        <v>71.273600000000002</v>
+        <v>64.337400000000002</v>
       </c>
       <c r="F96">
-        <v>74.714399999999998</v>
+        <v>64.954499999999996</v>
       </c>
       <c r="G96">
-        <v>74.696700000000007</v>
+        <v>60.048699999999997</v>
       </c>
       <c r="H96">
-        <v>72.732699999999994</v>
+        <v>61.807400000000001</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
@@ -3384,22 +3384,22 @@
         <v>109</v>
       </c>
       <c r="C97">
-        <v>328.48200000000003</v>
+        <v>299.20699999999999</v>
       </c>
       <c r="D97">
-        <v>330.83300000000003</v>
+        <v>310.91199999999998</v>
       </c>
       <c r="E97">
-        <v>358.31900000000002</v>
+        <v>342.64100000000002</v>
       </c>
       <c r="F97">
-        <v>332.16500000000002</v>
+        <v>310.197</v>
       </c>
       <c r="G97">
-        <v>368.07100000000003</v>
+        <v>334.60700000000003</v>
       </c>
       <c r="H97">
-        <v>357.61900000000003</v>
+        <v>332.899</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
@@ -3410,22 +3410,22 @@
         <v>109</v>
       </c>
       <c r="C98">
-        <v>365.303</v>
+        <v>337.82299999999998</v>
       </c>
       <c r="D98">
-        <v>367.589</v>
+        <v>347.755</v>
       </c>
       <c r="E98">
-        <v>386.88400000000001</v>
+        <v>371.286</v>
       </c>
       <c r="F98">
-        <v>370.91500000000002</v>
+        <v>350.73599999999999</v>
       </c>
       <c r="G98">
-        <v>396.33</v>
+        <v>362.97500000000002</v>
       </c>
       <c r="H98">
-        <v>385.57600000000002</v>
+        <v>360.916</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
@@ -3436,22 +3436,22 @@
         <v>17</v>
       </c>
       <c r="C99">
-        <v>2208.2199999999998</v>
+        <v>1724.21</v>
       </c>
       <c r="D99">
-        <v>2242.0500000000002</v>
+        <v>2027.57</v>
       </c>
       <c r="E99">
-        <v>6080.37</v>
+        <v>5344.13</v>
       </c>
       <c r="F99">
-        <v>2006.23</v>
+        <v>1651.43</v>
       </c>
       <c r="G99">
-        <v>6898.31</v>
+        <v>5253.01</v>
       </c>
       <c r="H99">
-        <v>6676.51</v>
+        <v>5430.46</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
@@ -3462,22 +3462,22 @@
         <v>109</v>
       </c>
       <c r="C100">
-        <v>240.48400000000001</v>
+        <v>214.90600000000001</v>
       </c>
       <c r="D100">
-        <v>242.386</v>
+        <v>220.14</v>
       </c>
       <c r="E100">
-        <v>241.63800000000001</v>
+        <v>225.99700000000001</v>
       </c>
       <c r="F100">
-        <v>242.834</v>
+        <v>223.22</v>
       </c>
       <c r="G100">
-        <v>249.77099999999999</v>
+        <v>217.05099999999999</v>
       </c>
       <c r="H100">
-        <v>243.10400000000001</v>
+        <v>218.66800000000001</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
@@ -3488,22 +3488,22 @@
         <v>17</v>
       </c>
       <c r="C101">
-        <v>1484.57</v>
+        <v>1120.19</v>
       </c>
       <c r="D101">
-        <v>1509.78</v>
+        <v>1310.81</v>
       </c>
       <c r="E101">
-        <v>3878.3</v>
+        <v>3322.08</v>
       </c>
       <c r="F101">
-        <v>1341.33</v>
+        <v>1073.3499999999999</v>
       </c>
       <c r="G101">
-        <v>4439.6499999999996</v>
+        <v>3208.04</v>
       </c>
       <c r="H101">
-        <v>4298.92</v>
+        <v>3360.17</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
@@ -3511,22 +3511,22 @@
         <v>116</v>
       </c>
       <c r="C102">
-        <v>0.76468400000000003</v>
+        <v>0.80057299999999998</v>
       </c>
       <c r="D102">
-        <v>0.76204499999999997</v>
+        <v>0.80086999999999997</v>
       </c>
       <c r="E102">
-        <v>0.810392</v>
+        <v>0.82788899999999999</v>
       </c>
       <c r="F102">
-        <v>0.77730399999999999</v>
+        <v>0.80338900000000002</v>
       </c>
       <c r="G102">
-        <v>0.80385499999999999</v>
+        <v>0.842055</v>
       </c>
       <c r="H102">
-        <v>0.80290700000000004</v>
+        <v>0.83123800000000003</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -3534,22 +3534,22 @@
         <v>117</v>
       </c>
       <c r="C103">
-        <v>0.72183299999999995</v>
+        <v>0.67408199999999996</v>
       </c>
       <c r="D103">
-        <v>0.72536100000000003</v>
+        <v>0.67449199999999998</v>
       </c>
       <c r="E103">
-        <v>0.66531399999999996</v>
+        <v>0.64257399999999998</v>
       </c>
       <c r="F103">
-        <v>0.70640400000000003</v>
+        <v>0.67071800000000004</v>
       </c>
       <c r="G103">
-        <v>0.67403100000000005</v>
+        <v>0.62423499999999998</v>
       </c>
       <c r="H103">
-        <v>0.67487900000000001</v>
+        <v>0.63779699999999995</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
@@ -3583,22 +3583,22 @@
         <v>119</v>
       </c>
       <c r="C105">
-        <v>0.30681399999999998</v>
+        <v>0.32017600000000002</v>
       </c>
       <c r="D105">
-        <v>0.30574000000000001</v>
+        <v>0.32102700000000001</v>
       </c>
       <c r="E105">
-        <v>0.326683</v>
+        <v>0.33420899999999998</v>
       </c>
       <c r="F105">
-        <v>0.31084600000000001</v>
+        <v>0.31997799999999998</v>
       </c>
       <c r="G105">
-        <v>0.32372200000000001</v>
+        <v>0.340337</v>
       </c>
       <c r="H105">
-        <v>0.32391399999999998</v>
+        <v>0.33603</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
@@ -3632,22 +3632,22 @@
         <v>121</v>
       </c>
       <c r="C107">
-        <v>0.25966499999999998</v>
+        <v>0.29060000000000002</v>
       </c>
       <c r="D107">
-        <v>0.25730399999999998</v>
+        <v>0.29417100000000002</v>
       </c>
       <c r="E107">
-        <v>0.31492999999999999</v>
+        <v>0.33529500000000001</v>
       </c>
       <c r="F107">
-        <v>0.26875700000000002</v>
+        <v>0.29088799999999998</v>
       </c>
       <c r="G107">
-        <v>0.30769000000000002</v>
+        <v>0.35350199999999998</v>
       </c>
       <c r="H107">
-        <v>0.30705199999999999</v>
+        <v>0.340055</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
@@ -3655,22 +3655,22 @@
         <v>122</v>
       </c>
       <c r="C108">
-        <v>0.42996499999999999</v>
+        <v>0.42941299999999999</v>
       </c>
       <c r="D108">
-        <v>0.42996600000000001</v>
+        <v>0.42963200000000001</v>
       </c>
       <c r="E108">
-        <v>0.430033</v>
+        <v>0.42999500000000002</v>
       </c>
       <c r="F108">
-        <v>0.43042599999999998</v>
+        <v>0.42965500000000001</v>
       </c>
       <c r="G108">
-        <v>0.430064</v>
+        <v>0.42993500000000001</v>
       </c>
       <c r="H108">
-        <v>0.43004199999999998</v>
+        <v>0.429921</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
@@ -3704,22 +3704,22 @@
         <v>124</v>
       </c>
       <c r="C110">
-        <v>3.5463300000000002</v>
+        <v>3.33081</v>
       </c>
       <c r="D110">
-        <v>3.5697700000000001</v>
+        <v>3.4009399999999999</v>
       </c>
       <c r="E110">
-        <v>2.9273400000000001</v>
+        <v>2.7451300000000001</v>
       </c>
       <c r="F110">
-        <v>3.7606799999999998</v>
+        <v>3.6401500000000002</v>
       </c>
       <c r="G110">
-        <v>2.5108100000000002</v>
+        <v>2.04528</v>
       </c>
       <c r="H110">
-        <v>2.4230700000000001</v>
+        <v>2.0469400000000002</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
@@ -3727,22 +3727,22 @@
         <v>125</v>
       </c>
       <c r="C111">
-        <v>5.3954399999999998</v>
+        <v>5.3332800000000002</v>
       </c>
       <c r="D111">
-        <v>5.4141500000000002</v>
+        <v>6.1410499999999999</v>
       </c>
       <c r="E111">
-        <v>5.1408399999999999</v>
+        <v>5.0257199999999997</v>
       </c>
       <c r="F111">
-        <v>6.4443999999999999</v>
+        <v>6.53939</v>
       </c>
       <c r="G111">
-        <v>2.9367999999999999</v>
+        <v>2.4595600000000002</v>
       </c>
       <c r="H111">
-        <v>2.4230700000000001</v>
+        <v>2.0469400000000002</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
@@ -3773,22 +3773,22 @@
         <v>127</v>
       </c>
       <c r="C113">
-        <v>5.0208500000000003</v>
+        <v>5.0381999999999998</v>
       </c>
       <c r="D113">
-        <v>5.0155900000000004</v>
+        <v>5.1186999999999996</v>
       </c>
       <c r="E113">
-        <v>5.3809800000000001</v>
+        <v>5.4391400000000001</v>
       </c>
       <c r="F113">
-        <v>4.9997199999999999</v>
+        <v>4.9942200000000003</v>
       </c>
       <c r="G113">
-        <v>5.36165</v>
+        <v>5.4932600000000003</v>
       </c>
       <c r="H113">
-        <v>5.3630599999999999</v>
+        <v>5.4582499999999996</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
@@ -3911,22 +3911,22 @@
         <v>133</v>
       </c>
       <c r="C119">
-        <v>1.9735100000000001</v>
+        <v>1.8590800000000001</v>
       </c>
       <c r="D119">
-        <v>1.9811399999999999</v>
+        <v>1.8577999999999999</v>
       </c>
       <c r="E119">
-        <v>1.8214900000000001</v>
+        <v>1.75993</v>
       </c>
       <c r="F119">
-        <v>1.93438</v>
+        <v>1.8464100000000001</v>
       </c>
       <c r="G119">
-        <v>1.84321</v>
+        <v>1.70695</v>
       </c>
       <c r="H119">
-        <v>1.8478600000000001</v>
+        <v>1.7486699999999999</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
@@ -3934,22 +3934,22 @@
         <v>134</v>
       </c>
       <c r="C120">
-        <v>2.0436800000000002</v>
+        <v>2.1972900000000002</v>
       </c>
       <c r="D120">
-        <v>2.0314100000000002</v>
+        <v>2.2066599999999998</v>
       </c>
       <c r="E120">
-        <v>2.2687499999999998</v>
+        <v>2.3565499999999999</v>
       </c>
       <c r="F120">
-        <v>2.0873300000000001</v>
+        <v>2.1954600000000002</v>
       </c>
       <c r="G120">
-        <v>2.23387</v>
+        <v>2.4287000000000001</v>
       </c>
       <c r="H120">
-        <v>2.23685</v>
+        <v>2.37873</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
@@ -4113,19 +4113,19 @@
         <v>141</v>
       </c>
       <c r="C127">
-        <v>0.511961</v>
+        <v>0.54718599999999995</v>
       </c>
       <c r="D127">
-        <v>0.50969699999999996</v>
+        <v>0.61842600000000003</v>
       </c>
       <c r="E127">
-        <v>0.60346</v>
+        <v>0.62561100000000003</v>
       </c>
       <c r="F127">
-        <v>0.58967899999999995</v>
+        <v>0.61582599999999998</v>
       </c>
       <c r="G127">
-        <v>0.25420399999999999</v>
+        <v>0.28900700000000001</v>
       </c>
       <c r="H127">
         <v>0</v>
@@ -4136,22 +4136,22 @@
         <v>142</v>
       </c>
       <c r="C128">
-        <v>0.48729</v>
+        <v>0.458258</v>
       </c>
       <c r="D128">
-        <v>0.488512</v>
+        <v>0.48049199999999997</v>
       </c>
       <c r="E128">
-        <v>0.46483000000000002</v>
+        <v>0.45096599999999998</v>
       </c>
       <c r="F128">
-        <v>0.49626700000000001</v>
+        <v>0.47253499999999998</v>
       </c>
       <c r="G128">
-        <v>0.428004</v>
+        <v>0.39637</v>
       </c>
       <c r="H128">
-        <v>0.42722700000000002</v>
+        <v>0.40289599999999998</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.25">
@@ -4182,22 +4182,22 @@
         <v>144</v>
       </c>
       <c r="C130">
-        <v>3.1958799999999998</v>
+        <v>2.6992500000000001</v>
       </c>
       <c r="D130">
-        <v>3.2277499999999999</v>
+        <v>2.6713499999999999</v>
       </c>
       <c r="E130">
-        <v>2.4796299999999998</v>
+        <v>2.2684199999999999</v>
       </c>
       <c r="F130">
-        <v>3.04271</v>
+        <v>2.6614399999999998</v>
       </c>
       <c r="G130">
-        <v>2.5627399999999998</v>
+        <v>2.1276799999999998</v>
       </c>
       <c r="H130">
-        <v>2.5787900000000001</v>
+        <v>2.2353100000000001</v>
       </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.25">
@@ -4208,7 +4208,7 @@
         <v>189.36199999999999</v>
       </c>
       <c r="D131">
-        <v>189.36199999999999</v>
+        <v>240.459</v>
       </c>
       <c r="E131">
         <v>386.42399999999998</v>
@@ -4228,22 +4228,22 @@
         <v>146</v>
       </c>
       <c r="C132">
-        <v>22430.9</v>
+        <v>21020.9</v>
       </c>
       <c r="D132">
-        <v>22534.1</v>
+        <v>21552.2</v>
       </c>
       <c r="E132">
-        <v>23535.4</v>
+        <v>22868.9</v>
       </c>
       <c r="F132">
-        <v>22373.3</v>
+        <v>21303.3</v>
       </c>
       <c r="G132">
-        <v>23921.5</v>
+        <v>22498.1</v>
       </c>
       <c r="H132">
-        <v>23577.599999999999</v>
+        <v>22518.3</v>
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.25">
@@ -4251,22 +4251,22 @@
         <v>147</v>
       </c>
       <c r="C133">
-        <v>0.98380999999999996</v>
+        <v>0.92196800000000001</v>
       </c>
       <c r="D133">
-        <v>0.98833700000000002</v>
+        <v>0.945272</v>
       </c>
       <c r="E133">
-        <v>1.03226</v>
+        <v>1.00302</v>
       </c>
       <c r="F133">
-        <v>0.98128599999999999</v>
+        <v>0.93435500000000005</v>
       </c>
       <c r="G133">
-        <v>1.0491900000000001</v>
+        <v>0.98675800000000002</v>
       </c>
       <c r="H133">
-        <v>1.0341</v>
+        <v>0.98764300000000005</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.25">
@@ -4274,22 +4274,22 @@
         <v>148</v>
       </c>
       <c r="C134">
-        <v>0.98932299999999995</v>
+        <v>0.94685299999999994</v>
       </c>
       <c r="D134">
-        <v>0.99232200000000004</v>
+        <v>0.951183</v>
       </c>
       <c r="E134">
-        <v>0.95526900000000003</v>
+        <v>0.93707700000000005</v>
       </c>
       <c r="F134">
-        <v>0.97215399999999996</v>
+        <v>0.94003800000000004</v>
       </c>
       <c r="G134">
-        <v>0.96213599999999999</v>
+        <v>0.92308000000000001</v>
       </c>
       <c r="H134">
-        <v>0.96365900000000004</v>
+        <v>0.93452000000000002</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.25">
@@ -4297,22 +4297,22 @@
         <v>149</v>
       </c>
       <c r="C135">
-        <v>23.055900000000001</v>
+        <v>26.787199999999999</v>
       </c>
       <c r="D135">
-        <v>23.278300000000002</v>
+        <v>27.742799999999999</v>
       </c>
       <c r="E135">
-        <v>31.7683</v>
+        <v>34.2956</v>
       </c>
       <c r="F135">
-        <v>24.288699999999999</v>
+        <v>26.9133</v>
       </c>
       <c r="G135">
-        <v>30.965299999999999</v>
+        <v>36.561399999999999</v>
       </c>
       <c r="H135">
-        <v>30.665700000000001</v>
+        <v>34.740400000000001</v>
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.25">
@@ -4320,22 +4320,22 @@
         <v>150</v>
       </c>
       <c r="C136">
-        <v>21.3292</v>
+        <v>24.611999999999998</v>
       </c>
       <c r="D136">
-        <v>20.988600000000002</v>
+        <v>25.663499999999999</v>
       </c>
       <c r="E136">
-        <v>29.249099999999999</v>
+        <v>30.499300000000002</v>
       </c>
       <c r="F136">
-        <v>22.646000000000001</v>
+        <v>24.266400000000001</v>
       </c>
       <c r="G136">
-        <v>28.5733</v>
+        <v>31.210899999999999</v>
       </c>
       <c r="H136">
-        <v>28.311399999999999</v>
+        <v>30.677399999999999</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.25">
@@ -4343,22 +4343,22 @@
         <v>151</v>
       </c>
       <c r="C137">
-        <v>9.8087400000000002</v>
+        <v>9.0398499999999995</v>
       </c>
       <c r="D137">
-        <v>9.8631700000000002</v>
+        <v>9.0366199999999992</v>
       </c>
       <c r="E137">
-        <v>8.8515700000000006</v>
+        <v>8.4967199999999998</v>
       </c>
       <c r="F137">
-        <v>9.5183900000000001</v>
+        <v>8.9468800000000002</v>
       </c>
       <c r="G137">
-        <v>8.9803599999999992</v>
+        <v>8.2118800000000007</v>
       </c>
       <c r="H137">
-        <v>9.0162800000000001</v>
+        <v>8.4427000000000003</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.25">
@@ -4366,22 +4366,22 @@
         <v>152</v>
       </c>
       <c r="C138">
-        <v>14244.8</v>
+        <v>12821.6</v>
       </c>
       <c r="D138">
-        <v>14345.8</v>
+        <v>13035.7</v>
       </c>
       <c r="E138">
-        <v>13781.5</v>
+        <v>13163.6</v>
       </c>
       <c r="F138">
-        <v>14046.4</v>
+        <v>12988</v>
       </c>
       <c r="G138">
-        <v>14085.6</v>
+        <v>12775</v>
       </c>
       <c r="H138">
-        <v>13906.5</v>
+        <v>12921.5</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.25">
@@ -4389,22 +4389,22 @@
         <v>153</v>
       </c>
       <c r="C139">
-        <v>0.97567400000000004</v>
+        <v>0.878193</v>
       </c>
       <c r="D139">
-        <v>0.98259099999999999</v>
+        <v>0.89285300000000001</v>
       </c>
       <c r="E139">
-        <v>0.94393800000000005</v>
+        <v>0.901617</v>
       </c>
       <c r="F139">
-        <v>0.96207900000000002</v>
+        <v>0.88958999999999999</v>
       </c>
       <c r="G139">
-        <v>0.96477000000000002</v>
+        <v>0.875</v>
       </c>
       <c r="H139">
-        <v>0.95249899999999998</v>
+        <v>0.88503100000000001</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.25">
@@ -4412,22 +4412,22 @@
         <v>154</v>
       </c>
       <c r="C140">
-        <v>0.97567400000000004</v>
+        <v>0.878193</v>
       </c>
       <c r="D140">
-        <v>0.98259099999999999</v>
+        <v>0.87336000000000003</v>
       </c>
       <c r="E140">
-        <v>0.840951</v>
+        <v>0.80324600000000002</v>
       </c>
       <c r="F140">
-        <v>0.94107499999999999</v>
+        <v>0.87016899999999997</v>
       </c>
       <c r="G140">
-        <v>0.85468100000000002</v>
+        <v>0.77515400000000001</v>
       </c>
       <c r="H140">
-        <v>0.85813799999999996</v>
+        <v>0.79735400000000001</v>
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.25">
@@ -4435,22 +4435,22 @@
         <v>155</v>
       </c>
       <c r="C141">
-        <v>2.4455900000000002</v>
+        <v>2.1684199999999998</v>
       </c>
       <c r="D141">
-        <v>2.46095</v>
+        <v>2.1470400000000001</v>
       </c>
       <c r="E141">
-        <v>2.0186700000000002</v>
+        <v>1.88948</v>
       </c>
       <c r="F141">
-        <v>2.3688099999999999</v>
+        <v>2.1457999999999999</v>
       </c>
       <c r="G141">
-        <v>2.0682999999999998</v>
+        <v>1.80487</v>
       </c>
       <c r="H141">
-        <v>2.07877</v>
+        <v>1.8700699999999999</v>
       </c>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.25">
@@ -4458,22 +4458,22 @@
         <v>156</v>
       </c>
       <c r="C142">
-        <v>46.556800000000003</v>
+        <v>48.885300000000001</v>
       </c>
       <c r="D142">
-        <v>46.280099999999997</v>
+        <v>50.531199999999998</v>
       </c>
       <c r="E142">
-        <v>57.8934</v>
+        <v>63.650799999999997</v>
       </c>
       <c r="F142">
-        <v>46.068199999999997</v>
+        <v>48.148499999999999</v>
       </c>
       <c r="G142">
-        <v>55.949800000000003</v>
+        <v>69.886799999999994</v>
       </c>
       <c r="H142">
-        <v>56.035800000000002</v>
+        <v>65.096800000000002</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.25">
@@ -4481,22 +4481,22 @@
         <v>157</v>
       </c>
       <c r="C143">
-        <v>23.457799999999999</v>
+        <v>24.492899999999999</v>
       </c>
       <c r="D143">
-        <v>23.4209</v>
+        <v>25.351199999999999</v>
       </c>
       <c r="E143">
-        <v>29.4786</v>
+        <v>33.150100000000002</v>
       </c>
       <c r="F143">
-        <v>23.0032</v>
+        <v>24.367799999999999</v>
       </c>
       <c r="G143">
-        <v>28.2501</v>
+        <v>36.461300000000001</v>
       </c>
       <c r="H143">
-        <v>28.1844</v>
+        <v>33.9758</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.25">
@@ -4504,22 +4504,22 @@
         <v>158</v>
       </c>
       <c r="C144">
-        <v>2.4455900000000002</v>
+        <v>2.1684199999999998</v>
       </c>
       <c r="D144">
-        <v>2.46095</v>
+        <v>2.1470400000000001</v>
       </c>
       <c r="E144">
-        <v>2.0186700000000002</v>
+        <v>1.88948</v>
       </c>
       <c r="F144">
-        <v>2.3688099999999999</v>
+        <v>2.1457999999999999</v>
       </c>
       <c r="G144">
-        <v>2.0682999999999998</v>
+        <v>1.80487</v>
       </c>
       <c r="H144">
-        <v>2.07877</v>
+        <v>1.8700699999999999</v>
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.25">
@@ -4527,22 +4527,22 @@
         <v>159</v>
       </c>
       <c r="C145">
-        <v>46.556800000000003</v>
+        <v>48.885300000000001</v>
       </c>
       <c r="D145">
-        <v>46.280099999999997</v>
+        <v>50.531199999999998</v>
       </c>
       <c r="E145">
-        <v>57.8934</v>
+        <v>63.650799999999997</v>
       </c>
       <c r="F145">
-        <v>46.068199999999997</v>
+        <v>48.148499999999999</v>
       </c>
       <c r="G145">
-        <v>55.949800000000003</v>
+        <v>69.886799999999994</v>
       </c>
       <c r="H145">
-        <v>56.035800000000002</v>
+        <v>65.096800000000002</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.25">
@@ -4550,22 +4550,22 @@
         <v>160</v>
       </c>
       <c r="C146">
-        <v>23.457799999999999</v>
+        <v>24.492899999999999</v>
       </c>
       <c r="D146">
-        <v>23.4209</v>
+        <v>25.351199999999999</v>
       </c>
       <c r="E146">
-        <v>29.4786</v>
+        <v>33.150100000000002</v>
       </c>
       <c r="F146">
-        <v>23.0032</v>
+        <v>24.367799999999999</v>
       </c>
       <c r="G146">
-        <v>28.2501</v>
+        <v>36.461300000000001</v>
       </c>
       <c r="H146">
-        <v>28.1844</v>
+        <v>33.9758</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.25">
@@ -4573,22 +4573,22 @@
         <v>161</v>
       </c>
       <c r="C147">
-        <v>2.04996</v>
+        <v>2.2756799999999999</v>
       </c>
       <c r="D147">
-        <v>2.0354399999999999</v>
+        <v>2.2603800000000001</v>
       </c>
       <c r="E147">
-        <v>2.2602799999999998</v>
+        <v>2.3737900000000001</v>
       </c>
       <c r="F147">
-        <v>2.12846</v>
+        <v>2.30436</v>
       </c>
       <c r="G147">
-        <v>2.21794</v>
+        <v>2.4690400000000001</v>
       </c>
       <c r="H147">
-        <v>2.2140599999999999</v>
+        <v>2.3952300000000002</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.25">
@@ -4596,22 +4596,22 @@
         <v>162</v>
       </c>
       <c r="C148">
-        <v>0.99423600000000001</v>
+        <v>0.96291199999999999</v>
       </c>
       <c r="D148">
-        <v>0.99594800000000006</v>
+        <v>0.97666200000000003</v>
       </c>
       <c r="E148">
-        <v>1.02024</v>
+        <v>1.0107299999999999</v>
       </c>
       <c r="F148">
-        <v>0.98125499999999999</v>
+        <v>0.95519100000000001</v>
       </c>
       <c r="G148">
-        <v>1.0249600000000001</v>
+        <v>1.0050399999999999</v>
       </c>
       <c r="H148">
-        <v>1.0241199999999999</v>
+        <v>1.00936</v>
       </c>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.25">
@@ -4622,22 +4622,22 @@
         <v>15</v>
       </c>
       <c r="C149">
-        <v>2.2438099999999999</v>
+        <v>2.1730700000000001</v>
       </c>
       <c r="D149">
-        <v>2.2476400000000001</v>
+        <v>2.2056200000000001</v>
       </c>
       <c r="E149">
-        <v>2.3024300000000002</v>
+        <v>2.28186</v>
       </c>
       <c r="F149">
-        <v>2.2127500000000002</v>
+        <v>2.1538599999999999</v>
       </c>
       <c r="G149">
-        <v>2.31264</v>
+        <v>2.26952</v>
       </c>
       <c r="H149">
-        <v>2.3108300000000002</v>
+        <v>2.2788900000000001</v>
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.25">
@@ -4645,22 +4645,22 @@
         <v>164</v>
       </c>
       <c r="C150">
-        <v>0.98636100000000004</v>
+        <v>0.91764299999999999</v>
       </c>
       <c r="D150">
-        <v>0.99041900000000005</v>
+        <v>0.92328299999999996</v>
       </c>
       <c r="E150">
-        <v>0.93365699999999996</v>
+        <v>0.909914</v>
       </c>
       <c r="F150">
-        <v>0.96111199999999997</v>
+        <v>0.90823399999999999</v>
       </c>
       <c r="G150">
-        <v>0.94273099999999999</v>
+        <v>0.89289499999999999</v>
       </c>
       <c r="H150">
-        <v>0.94422399999999995</v>
+        <v>0.90651099999999996</v>
       </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.25">
@@ -4671,22 +4671,22 @@
         <v>15</v>
       </c>
       <c r="C151">
-        <v>5.9476199999999997</v>
+        <v>5.5319399999999996</v>
       </c>
       <c r="D151">
-        <v>5.9719899999999999</v>
+        <v>5.5708700000000002</v>
       </c>
       <c r="E151">
-        <v>5.67584</v>
+        <v>5.5268899999999999</v>
       </c>
       <c r="F151">
-        <v>5.7906700000000004</v>
+        <v>5.4692499999999997</v>
       </c>
       <c r="G151">
-        <v>5.7311800000000002</v>
+        <v>5.4238900000000001</v>
       </c>
       <c r="H151">
-        <v>5.7408599999999996</v>
+        <v>5.5086899999999996</v>
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
@@ -4717,22 +4717,22 @@
         <v>167</v>
       </c>
       <c r="C153">
-        <v>3.1958799999999998</v>
+        <v>2.6992500000000001</v>
       </c>
       <c r="D153">
-        <v>3.2277499999999999</v>
+        <v>2.6713499999999999</v>
       </c>
       <c r="E153">
-        <v>2.4796299999999998</v>
+        <v>2.2684199999999999</v>
       </c>
       <c r="F153">
-        <v>3.04271</v>
+        <v>2.6614399999999998</v>
       </c>
       <c r="G153">
-        <v>2.5627399999999998</v>
+        <v>2.1276799999999998</v>
       </c>
       <c r="H153">
-        <v>2.5787900000000001</v>
+        <v>2.2353100000000001</v>
       </c>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.25">
@@ -4740,22 +4740,22 @@
         <v>168</v>
       </c>
       <c r="C154">
-        <v>98.275000000000006</v>
+        <v>94.126900000000006</v>
       </c>
       <c r="D154">
-        <v>98.732299999999995</v>
+        <v>94.057900000000004</v>
       </c>
       <c r="E154">
-        <v>94.874700000000004</v>
+        <v>91.442800000000005</v>
       </c>
       <c r="F154">
-        <v>100.015</v>
+        <v>97.440799999999996</v>
       </c>
       <c r="G154">
-        <v>96.768100000000004</v>
+        <v>89.2483</v>
       </c>
       <c r="H154">
-        <v>94.825699999999998</v>
+        <v>89.305300000000003</v>
       </c>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.25">
@@ -4927,16 +4927,16 @@
         <v>176</v>
       </c>
       <c r="C162">
-        <v>0.98863199999999996</v>
+        <v>0.98710500000000001</v>
       </c>
       <c r="D162">
-        <v>0.98868699999999998</v>
+        <v>0.98918899999999998</v>
       </c>
       <c r="E162">
         <v>1</v>
       </c>
       <c r="F162">
-        <v>0.98634100000000002</v>
+        <v>0.98499000000000003</v>
       </c>
       <c r="G162">
         <v>1</v>
@@ -4950,16 +4950,16 @@
         <v>177</v>
       </c>
       <c r="C163">
-        <v>0.99431599999999998</v>
+        <v>0.99355300000000002</v>
       </c>
       <c r="D163">
-        <v>0.99434400000000001</v>
+        <v>0.99459399999999998</v>
       </c>
       <c r="E163">
         <v>1</v>
       </c>
       <c r="F163">
-        <v>0.99317</v>
+        <v>0.99249500000000002</v>
       </c>
       <c r="G163">
         <v>1</v>
@@ -4973,16 +4973,16 @@
         <v>178</v>
       </c>
       <c r="C164">
-        <v>0.99792899999999995</v>
+        <v>0.99518399999999996</v>
       </c>
       <c r="D164">
-        <v>0.99804199999999998</v>
+        <v>0.99775599999999998</v>
       </c>
       <c r="E164">
         <v>1</v>
       </c>
       <c r="F164">
-        <v>0.99523200000000001</v>
+        <v>0.99284600000000001</v>
       </c>
       <c r="G164">
         <v>1</v>
@@ -4996,16 +4996,16 @@
         <v>179</v>
       </c>
       <c r="C165">
-        <v>0.99896399999999996</v>
+        <v>0.99759200000000003</v>
       </c>
       <c r="D165">
-        <v>0.99902100000000005</v>
+        <v>0.99887800000000004</v>
       </c>
       <c r="E165">
         <v>1</v>
       </c>
       <c r="F165">
-        <v>0.99761599999999995</v>
+        <v>0.99642299999999995</v>
       </c>
       <c r="G165">
         <v>1</v>
@@ -5019,19 +5019,19 @@
         <v>180</v>
       </c>
       <c r="C166">
-        <v>0.98037399999999997</v>
+        <v>0.97763800000000001</v>
       </c>
       <c r="D166">
-        <v>0.98048599999999997</v>
+        <v>0.98021400000000003</v>
       </c>
       <c r="E166">
-        <v>1</v>
+        <v>0.99900500000000003</v>
       </c>
       <c r="F166">
-        <v>0.97764200000000001</v>
+        <v>0.97525200000000001</v>
       </c>
       <c r="G166">
-        <v>1</v>
+        <v>0.99943400000000004</v>
       </c>
       <c r="H166">
         <v>1</v>
@@ -5042,19 +5042,19 @@
         <v>181</v>
       </c>
       <c r="C167">
-        <v>0.99018700000000004</v>
+        <v>0.988819</v>
       </c>
       <c r="D167">
-        <v>0.99024299999999998</v>
+        <v>0.99010699999999996</v>
       </c>
       <c r="E167">
-        <v>1</v>
+        <v>0.99950300000000003</v>
       </c>
       <c r="F167">
-        <v>0.98882099999999995</v>
+        <v>0.987626</v>
       </c>
       <c r="G167">
-        <v>1</v>
+        <v>0.99971699999999997</v>
       </c>
       <c r="H167">
         <v>1</v>
@@ -5091,22 +5091,22 @@
         <v>184</v>
       </c>
       <c r="C169">
-        <v>0.50026199999999998</v>
+        <v>0.52122100000000005</v>
       </c>
       <c r="D169">
-        <v>0.49991200000000002</v>
+        <v>0.50372399999999995</v>
       </c>
       <c r="E169">
-        <v>0.45402399999999998</v>
+        <v>0.455876</v>
       </c>
       <c r="F169">
-        <v>0.51042900000000002</v>
+        <v>0.53053700000000004</v>
       </c>
       <c r="G169">
-        <v>0.45197999999999999</v>
+        <v>0.45567200000000002</v>
       </c>
       <c r="H169">
-        <v>0.45282299999999998</v>
+        <v>0.45540999999999998</v>
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.25">
@@ -5117,22 +5117,22 @@
         <v>184</v>
       </c>
       <c r="C170">
-        <v>1566.55</v>
+        <v>1467.32</v>
       </c>
       <c r="D170">
-        <v>1575.58</v>
+        <v>1497.91</v>
       </c>
       <c r="E170">
-        <v>1630.98</v>
+        <v>1568.7</v>
       </c>
       <c r="F170">
-        <v>1599.96</v>
+        <v>1531.4</v>
       </c>
       <c r="G170">
-        <v>1669.45</v>
+        <v>1534.86</v>
       </c>
       <c r="H170">
-        <v>1624.79</v>
+        <v>1525.09</v>
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.25">
@@ -5143,22 +5143,22 @@
         <v>184</v>
       </c>
       <c r="C171">
-        <v>0.49123299999999998</v>
+        <v>0.475356</v>
       </c>
       <c r="D171">
-        <v>0.49351899999999999</v>
+        <v>0.46635900000000002</v>
       </c>
       <c r="E171">
-        <v>0.433195</v>
+        <v>0.41526800000000003</v>
       </c>
       <c r="F171">
-        <v>0.49017500000000003</v>
+        <v>0.48183199999999998</v>
       </c>
       <c r="G171">
-        <v>0.43953199999999998</v>
+        <v>0.39812199999999998</v>
       </c>
       <c r="H171">
-        <v>0.43809999999999999</v>
+        <v>0.40976899999999999</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.25">
@@ -5169,22 +5169,22 @@
         <v>184</v>
       </c>
       <c r="C172">
-        <v>0.97567400000000004</v>
+        <v>0.878193</v>
       </c>
       <c r="D172">
-        <v>0.98259099999999999</v>
+        <v>0.89285300000000001</v>
       </c>
       <c r="E172">
-        <v>0.94393800000000005</v>
+        <v>0.901617</v>
       </c>
       <c r="F172">
-        <v>0.96207900000000002</v>
+        <v>0.88958999999999999</v>
       </c>
       <c r="G172">
-        <v>0.96477000000000002</v>
+        <v>0.875</v>
       </c>
       <c r="H172">
-        <v>0.95249899999999998</v>
+        <v>0.88503100000000001</v>
       </c>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.25">
@@ -5195,22 +5195,22 @@
         <v>184</v>
       </c>
       <c r="C173">
-        <v>2.04996</v>
+        <v>2.2756799999999999</v>
       </c>
       <c r="D173">
-        <v>2.0354399999999999</v>
+        <v>2.2603800000000001</v>
       </c>
       <c r="E173">
-        <v>2.2602799999999998</v>
+        <v>2.3737900000000001</v>
       </c>
       <c r="F173">
-        <v>2.12846</v>
+        <v>2.30436</v>
       </c>
       <c r="G173">
-        <v>2.21794</v>
+        <v>2.4690400000000001</v>
       </c>
       <c r="H173">
-        <v>2.2140599999999999</v>
+        <v>2.3952300000000002</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.25">
@@ -5221,22 +5221,22 @@
         <v>184</v>
       </c>
       <c r="C174">
-        <v>0.50175400000000003</v>
+        <v>0.50917599999999996</v>
       </c>
       <c r="D174">
-        <v>0.50124800000000003</v>
+        <v>0.50646599999999997</v>
       </c>
       <c r="E174">
-        <v>0.50597400000000003</v>
+        <v>0.50726800000000005</v>
       </c>
       <c r="F174">
-        <v>0.50339100000000003</v>
+        <v>0.50875899999999996</v>
       </c>
       <c r="G174">
-        <v>0.50475899999999996</v>
+        <v>0.50862099999999999</v>
       </c>
       <c r="H174">
-        <v>0.50579499999999999</v>
+        <v>0.50876999999999994</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.25">
@@ -5247,22 +5247,22 @@
         <v>184</v>
       </c>
       <c r="C175">
-        <v>0.493168</v>
+        <v>0.46370699999999998</v>
       </c>
       <c r="D175">
-        <v>0.495139</v>
+        <v>0.461169</v>
       </c>
       <c r="E175">
-        <v>0.43689800000000001</v>
+        <v>0.420541</v>
       </c>
       <c r="F175">
-        <v>0.48285800000000001</v>
+        <v>0.46068599999999998</v>
       </c>
       <c r="G175">
-        <v>0.44252000000000002</v>
+        <v>0.41074699999999997</v>
       </c>
       <c r="H175">
-        <v>0.444635</v>
+        <v>0.41838500000000001</v>
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.25">
@@ -5276,7 +5276,7 @@
         <v>2.4606900000000001E-8</v>
       </c>
       <c r="D176">
-        <v>2.4606900000000001E-8</v>
+        <v>-5.9300799999999999E-7</v>
       </c>
       <c r="E176">
         <v>-4.5762299999999999E-6</v>

</xml_diff>